<commit_message>
feat: add flags to disable Excel report and GDrive sync, and update Excel database to true file
</commit_message>
<xml_diff>
--- a/HV_Mau 2_Tong hop KQRL cua SV.xlsx
+++ b/HV_Mau 2_Tong hop KQRL cua SV.xlsx
@@ -678,18 +678,12 @@
       <name val="Times New Roman"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE599"/>
-        <bgColor rgb="FFFFE599"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="26">
@@ -934,7 +928,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="68">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1034,7 +1028,7 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="20" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="17" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1042,46 +1036,19 @@
     <xf borderId="17" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="16" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="17" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="18" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="18" fillId="2" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="18" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="18" fillId="2" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="19" fillId="2" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="20" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="17" fillId="2" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="18" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="17" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="17" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="20" fillId="2" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf borderId="20" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="17" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="18" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="20" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="17" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1091,7 +1058,7 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="20" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="21" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1115,7 +1082,7 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="25" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
@@ -1945,42 +1912,42 @@
       <c r="Z17" s="24"/>
     </row>
     <row r="18">
-      <c r="A18" s="43">
+      <c r="A18" s="33">
         <v>5.0</v>
       </c>
-      <c r="B18" s="44" t="s">
+      <c r="B18" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="45" t="s">
+      <c r="C18" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="46" t="s">
+      <c r="D18" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="47">
+      <c r="E18" s="37">
         <v>17.0</v>
       </c>
-      <c r="F18" s="47">
+      <c r="F18" s="37">
         <v>19.0</v>
       </c>
-      <c r="G18" s="47">
-        <v>3.0</v>
-      </c>
-      <c r="H18" s="47">
+      <c r="G18" s="37">
+        <v>13.0</v>
+      </c>
+      <c r="H18" s="37">
         <v>18.0</v>
       </c>
-      <c r="I18" s="47">
+      <c r="I18" s="37">
         <v>0.0</v>
       </c>
-      <c r="J18" s="48">
+      <c r="J18" s="38">
         <f t="shared" si="1"/>
-        <v>57</v>
-      </c>
-      <c r="K18" s="49" t="str">
+        <v>67</v>
+      </c>
+      <c r="K18" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Trung bình</v>
-      </c>
-      <c r="L18" s="50"/>
+        <v>Khá</v>
+      </c>
+      <c r="L18" s="40"/>
       <c r="M18" s="24"/>
       <c r="N18" s="24"/>
       <c r="O18" s="24"/>
@@ -2049,42 +2016,42 @@
       <c r="Z19" s="24"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="43">
+      <c r="A20" s="33">
         <v>7.0</v>
       </c>
-      <c r="B20" s="44" t="s">
+      <c r="B20" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="45" t="s">
+      <c r="C20" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="46" t="s">
+      <c r="D20" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="47">
-        <v>14.0</v>
-      </c>
-      <c r="F20" s="47">
-        <v>20.0</v>
-      </c>
-      <c r="G20" s="47">
+      <c r="E20" s="37">
+        <v>16.0</v>
+      </c>
+      <c r="F20" s="37">
+        <v>23.0</v>
+      </c>
+      <c r="G20" s="37">
         <v>3.0</v>
       </c>
-      <c r="H20" s="47">
+      <c r="H20" s="37">
         <v>23.0</v>
       </c>
-      <c r="I20" s="47">
+      <c r="I20" s="37">
         <v>0.0</v>
       </c>
-      <c r="J20" s="48">
+      <c r="J20" s="38">
         <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="K20" s="49" t="str">
+        <v>65</v>
+      </c>
+      <c r="K20" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Trung bình</v>
-      </c>
-      <c r="L20" s="50"/>
+        <v>Khá</v>
+      </c>
+      <c r="L20" s="40"/>
       <c r="M20" s="24"/>
       <c r="N20" s="24"/>
       <c r="O20" s="24"/>
@@ -2413,42 +2380,42 @@
       <c r="Z26" s="24"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="43">
+      <c r="A27" s="33">
         <v>14.0</v>
       </c>
-      <c r="B27" s="51" t="s">
+      <c r="B27" s="42" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="45" t="s">
+      <c r="C27" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="46" t="s">
+      <c r="D27" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="E27" s="47">
+      <c r="E27" s="37">
         <v>14.0</v>
       </c>
-      <c r="F27" s="47">
+      <c r="F27" s="37">
         <v>20.0</v>
       </c>
-      <c r="G27" s="47">
-        <v>3.0</v>
-      </c>
-      <c r="H27" s="47">
+      <c r="G27" s="37">
+        <v>8.0</v>
+      </c>
+      <c r="H27" s="37">
         <v>23.0</v>
       </c>
-      <c r="I27" s="47">
+      <c r="I27" s="37">
         <v>0.0</v>
       </c>
-      <c r="J27" s="48">
+      <c r="J27" s="38">
         <f t="shared" si="1"/>
-        <v>60</v>
-      </c>
-      <c r="K27" s="49" t="str">
+        <v>65</v>
+      </c>
+      <c r="K27" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Trung bình</v>
-      </c>
-      <c r="L27" s="50"/>
+        <v>Khá</v>
+      </c>
+      <c r="L27" s="40"/>
       <c r="M27" s="24"/>
       <c r="N27" s="24"/>
       <c r="O27" s="24"/>
@@ -2544,7 +2511,7 @@
       <c r="I29" s="37">
         <v>3.0</v>
       </c>
-      <c r="J29" s="52">
+      <c r="J29" s="43">
         <f t="shared" si="1"/>
         <v>76.5</v>
       </c>
@@ -2725,42 +2692,42 @@
       <c r="Z32" s="24"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="43">
+      <c r="A33" s="33">
         <v>20.0</v>
       </c>
-      <c r="B33" s="53" t="s">
+      <c r="B33" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="C33" s="45" t="s">
+      <c r="C33" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="D33" s="46" t="s">
+      <c r="D33" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="E33" s="47">
+      <c r="E33" s="37">
         <v>17.0</v>
       </c>
-      <c r="F33" s="47">
+      <c r="F33" s="37">
         <v>20.0</v>
       </c>
-      <c r="G33" s="47">
-        <v>4.0</v>
-      </c>
-      <c r="H33" s="47">
+      <c r="G33" s="37">
+        <v>8.0</v>
+      </c>
+      <c r="H33" s="37">
         <v>23.0</v>
       </c>
-      <c r="I33" s="47">
+      <c r="I33" s="37">
         <v>0.0</v>
       </c>
-      <c r="J33" s="48">
+      <c r="J33" s="38">
         <f t="shared" si="1"/>
-        <v>64</v>
-      </c>
-      <c r="K33" s="49" t="str">
+        <v>68</v>
+      </c>
+      <c r="K33" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Trung bình</v>
-      </c>
-      <c r="L33" s="54"/>
+        <v>Khá</v>
+      </c>
+      <c r="L33" s="45"/>
       <c r="M33" s="24"/>
       <c r="N33" s="24"/>
       <c r="O33" s="24"/>
@@ -2832,7 +2799,7 @@
       <c r="A35" s="33">
         <v>22.0</v>
       </c>
-      <c r="B35" s="55" t="s">
+      <c r="B35" s="46" t="s">
         <v>86</v>
       </c>
       <c r="C35" s="35" t="s">
@@ -2841,20 +2808,30 @@
       <c r="D35" s="36" t="s">
         <v>88</v>
       </c>
-      <c r="E35" s="37"/>
-      <c r="F35" s="56"/>
-      <c r="G35" s="56"/>
-      <c r="H35" s="56"/>
-      <c r="I35" s="56"/>
+      <c r="E35" s="37">
+        <v>14.0</v>
+      </c>
+      <c r="F35" s="37">
+        <v>23.0</v>
+      </c>
+      <c r="G35" s="37">
+        <v>6.0</v>
+      </c>
+      <c r="H35" s="37">
+        <v>22.0</v>
+      </c>
+      <c r="I35" s="37">
+        <v>0.0</v>
+      </c>
       <c r="J35" s="38">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="K35" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Kém</v>
-      </c>
-      <c r="L35" s="40"/>
+        <v>Khá</v>
+      </c>
+      <c r="L35" s="47"/>
       <c r="M35" s="24"/>
       <c r="N35" s="24"/>
       <c r="O35" s="24"/>
@@ -2874,7 +2851,7 @@
       <c r="A36" s="33">
         <v>23.0</v>
       </c>
-      <c r="B36" s="55" t="s">
+      <c r="B36" s="46" t="s">
         <v>89</v>
       </c>
       <c r="C36" s="35" t="s">
@@ -2926,7 +2903,7 @@
       <c r="A37" s="33">
         <v>24.0</v>
       </c>
-      <c r="B37" s="57" t="s">
+      <c r="B37" s="48" t="s">
         <v>92</v>
       </c>
       <c r="C37" s="35" t="s">
@@ -2950,7 +2927,7 @@
       <c r="I37" s="37">
         <v>0.0</v>
       </c>
-      <c r="J37" s="58">
+      <c r="J37" s="49">
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
@@ -2958,7 +2935,7 @@
         <f t="shared" si="2"/>
         <v>Khá</v>
       </c>
-      <c r="L37" s="59"/>
+      <c r="L37" s="50"/>
       <c r="M37" s="24"/>
       <c r="N37" s="24"/>
       <c r="O37" s="24"/>
@@ -3027,42 +3004,42 @@
       <c r="Z38" s="24"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="43">
+      <c r="A39" s="33">
         <v>26.0</v>
       </c>
-      <c r="B39" s="44" t="s">
+      <c r="B39" s="41" t="s">
         <v>97</v>
       </c>
-      <c r="C39" s="45" t="s">
+      <c r="C39" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="D39" s="46" t="s">
+      <c r="D39" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="E39" s="47">
+      <c r="E39" s="37">
         <v>14.0</v>
       </c>
-      <c r="F39" s="47">
+      <c r="F39" s="37">
         <v>20.0</v>
       </c>
-      <c r="G39" s="47">
-        <v>7.0</v>
-      </c>
-      <c r="H39" s="47">
+      <c r="G39" s="37">
+        <v>9.0</v>
+      </c>
+      <c r="H39" s="37">
         <v>23.0</v>
       </c>
-      <c r="I39" s="47">
+      <c r="I39" s="37">
         <v>0.0</v>
       </c>
-      <c r="J39" s="48">
+      <c r="J39" s="38">
         <f t="shared" si="1"/>
-        <v>64</v>
-      </c>
-      <c r="K39" s="49" t="str">
+        <v>66</v>
+      </c>
+      <c r="K39" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Trung bình</v>
-      </c>
-      <c r="L39" s="54"/>
+        <v>Khá</v>
+      </c>
+      <c r="L39" s="45"/>
       <c r="M39" s="24"/>
       <c r="N39" s="24"/>
       <c r="O39" s="24"/>
@@ -3079,42 +3056,42 @@
       <c r="Z39" s="24"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="43">
+      <c r="A40" s="33">
         <v>27.0</v>
       </c>
-      <c r="B40" s="44" t="s">
+      <c r="B40" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="C40" s="45" t="s">
+      <c r="C40" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="D40" s="46" t="s">
+      <c r="D40" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="E40" s="47">
+      <c r="E40" s="37">
         <v>14.0</v>
       </c>
-      <c r="F40" s="47">
+      <c r="F40" s="37">
         <v>20.0</v>
       </c>
-      <c r="G40" s="47">
-        <v>5.0</v>
-      </c>
-      <c r="H40" s="47">
+      <c r="G40" s="37">
+        <v>9.0</v>
+      </c>
+      <c r="H40" s="37">
         <v>23.0</v>
       </c>
-      <c r="I40" s="47">
+      <c r="I40" s="37">
         <v>0.0</v>
       </c>
-      <c r="J40" s="48">
+      <c r="J40" s="38">
         <f t="shared" si="1"/>
-        <v>62</v>
-      </c>
-      <c r="K40" s="49" t="str">
+        <v>66</v>
+      </c>
+      <c r="K40" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Trung bình</v>
-      </c>
-      <c r="L40" s="50"/>
+        <v>Khá</v>
+      </c>
+      <c r="L40" s="40"/>
       <c r="M40" s="24"/>
       <c r="N40" s="24"/>
       <c r="O40" s="24"/>
@@ -3195,20 +3172,30 @@
       <c r="D42" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="E42" s="37"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="56"/>
-      <c r="H42" s="56"/>
-      <c r="I42" s="56"/>
+      <c r="E42" s="37">
+        <v>14.0</v>
+      </c>
+      <c r="F42" s="37">
+        <v>23.0</v>
+      </c>
+      <c r="G42" s="37">
+        <v>6.0</v>
+      </c>
+      <c r="H42" s="37">
+        <v>22.0</v>
+      </c>
+      <c r="I42" s="37">
+        <v>0.0</v>
+      </c>
       <c r="J42" s="38">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="K42" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Kém</v>
-      </c>
-      <c r="L42" s="40"/>
+        <v>Khá</v>
+      </c>
+      <c r="L42" s="47"/>
       <c r="M42" s="24"/>
       <c r="N42" s="24"/>
       <c r="O42" s="24"/>
@@ -3416,7 +3403,7 @@
         <f t="shared" si="2"/>
         <v>Tốt</v>
       </c>
-      <c r="L46" s="40"/>
+      <c r="L46" s="47"/>
       <c r="M46" s="24"/>
       <c r="N46" s="24"/>
       <c r="O46" s="24"/>
@@ -3433,42 +3420,42 @@
       <c r="Z46" s="24"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="43">
+      <c r="A47" s="33">
         <v>34.0</v>
       </c>
-      <c r="B47" s="44" t="s">
+      <c r="B47" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="C47" s="45" t="s">
+      <c r="C47" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="D47" s="46" t="s">
+      <c r="D47" s="36" t="s">
         <v>121</v>
       </c>
-      <c r="E47" s="47">
+      <c r="E47" s="37">
         <v>15.0</v>
       </c>
-      <c r="F47" s="47">
+      <c r="F47" s="37">
         <v>19.0</v>
       </c>
-      <c r="G47" s="47">
-        <v>7.0</v>
-      </c>
-      <c r="H47" s="47">
+      <c r="G47" s="37">
+        <v>8.0</v>
+      </c>
+      <c r="H47" s="37">
         <v>23.0</v>
       </c>
-      <c r="I47" s="47">
+      <c r="I47" s="37">
         <v>0.0</v>
       </c>
-      <c r="J47" s="48">
+      <c r="J47" s="38">
         <f t="shared" si="1"/>
-        <v>64</v>
-      </c>
-      <c r="K47" s="49" t="str">
+        <v>65</v>
+      </c>
+      <c r="K47" s="39" t="str">
         <f t="shared" si="2"/>
-        <v>Trung bình</v>
-      </c>
-      <c r="L47" s="50"/>
+        <v>Khá</v>
+      </c>
+      <c r="L47" s="40"/>
       <c r="M47" s="24"/>
       <c r="N47" s="24"/>
       <c r="O47" s="24"/>
@@ -3488,7 +3475,7 @@
       <c r="A48" s="33">
         <v>35.0</v>
       </c>
-      <c r="B48" s="55" t="s">
+      <c r="B48" s="46" t="s">
         <v>122</v>
       </c>
       <c r="C48" s="35" t="s">
@@ -3589,42 +3576,42 @@
       <c r="Z49" s="24"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="60">
+      <c r="A50" s="51">
         <v>37.0</v>
       </c>
-      <c r="B50" s="61" t="s">
+      <c r="B50" s="52" t="s">
         <v>127</v>
       </c>
-      <c r="C50" s="62" t="s">
+      <c r="C50" s="53" t="s">
         <v>101</v>
       </c>
-      <c r="D50" s="63" t="s">
+      <c r="D50" s="54" t="s">
         <v>128</v>
       </c>
-      <c r="E50" s="64">
+      <c r="E50" s="55">
         <v>17.0</v>
       </c>
-      <c r="F50" s="64">
+      <c r="F50" s="55">
         <v>23.0</v>
       </c>
-      <c r="G50" s="64">
+      <c r="G50" s="55">
         <v>16.0</v>
       </c>
-      <c r="H50" s="64">
+      <c r="H50" s="55">
         <v>23.0</v>
       </c>
-      <c r="I50" s="64">
+      <c r="I50" s="55">
         <v>7.0</v>
       </c>
-      <c r="J50" s="65">
+      <c r="J50" s="56">
         <f t="shared" si="1"/>
         <v>86</v>
       </c>
-      <c r="K50" s="66" t="str">
+      <c r="K50" s="57" t="str">
         <f t="shared" si="2"/>
         <v>Tốt</v>
       </c>
-      <c r="L50" s="67"/>
+      <c r="L50" s="58"/>
       <c r="M50" s="24"/>
       <c r="N50" s="24"/>
       <c r="O50" s="24"/>
@@ -3641,7 +3628,7 @@
       <c r="Z50" s="24"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="68"/>
+      <c r="A51" s="59"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -3669,299 +3656,299 @@
       <c r="Z51" s="3"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="69"/>
-      <c r="B52" s="70" t="s">
+      <c r="A52" s="60"/>
+      <c r="B52" s="61" t="s">
         <v>129</v>
       </c>
-      <c r="C52" s="69">
+      <c r="C52" s="60">
         <f>COUNTA($K$14:$K$50)</f>
         <v>37</v>
       </c>
-      <c r="D52" s="69" t="s">
+      <c r="D52" s="60" t="s">
         <v>130</v>
       </c>
-      <c r="E52" s="69"/>
-      <c r="F52" s="69"/>
-      <c r="G52" s="69"/>
-      <c r="H52" s="69"/>
-      <c r="I52" s="69"/>
-      <c r="J52" s="69"/>
-      <c r="K52" s="71"/>
-      <c r="L52" s="69"/>
-      <c r="M52" s="69"/>
-      <c r="N52" s="69"/>
-      <c r="O52" s="69"/>
-      <c r="P52" s="69"/>
-      <c r="Q52" s="69"/>
-      <c r="R52" s="69"/>
-      <c r="S52" s="69"/>
-      <c r="T52" s="69"/>
-      <c r="U52" s="69"/>
-      <c r="V52" s="69"/>
-      <c r="W52" s="69"/>
-      <c r="X52" s="69"/>
-      <c r="Y52" s="69"/>
-      <c r="Z52" s="69"/>
+      <c r="E52" s="60"/>
+      <c r="F52" s="60"/>
+      <c r="G52" s="60"/>
+      <c r="H52" s="60"/>
+      <c r="I52" s="60"/>
+      <c r="J52" s="60"/>
+      <c r="K52" s="62"/>
+      <c r="L52" s="60"/>
+      <c r="M52" s="60"/>
+      <c r="N52" s="60"/>
+      <c r="O52" s="60"/>
+      <c r="P52" s="60"/>
+      <c r="Q52" s="60"/>
+      <c r="R52" s="60"/>
+      <c r="S52" s="60"/>
+      <c r="T52" s="60"/>
+      <c r="U52" s="60"/>
+      <c r="V52" s="60"/>
+      <c r="W52" s="60"/>
+      <c r="X52" s="60"/>
+      <c r="Y52" s="60"/>
+      <c r="Z52" s="60"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="69" t="s">
+      <c r="A53" s="60" t="s">
         <v>131</v>
       </c>
-      <c r="B53" s="70"/>
-      <c r="C53" s="69"/>
-      <c r="D53" s="69"/>
-      <c r="E53" s="69"/>
-      <c r="F53" s="69"/>
-      <c r="G53" s="69"/>
-      <c r="H53" s="69"/>
-      <c r="I53" s="69"/>
-      <c r="J53" s="69"/>
-      <c r="K53" s="69"/>
-      <c r="L53" s="69"/>
-      <c r="M53" s="69"/>
-      <c r="N53" s="69"/>
-      <c r="O53" s="69"/>
-      <c r="P53" s="69"/>
-      <c r="Q53" s="69"/>
-      <c r="R53" s="69"/>
-      <c r="S53" s="69"/>
-      <c r="T53" s="69"/>
-      <c r="U53" s="69"/>
-      <c r="V53" s="69"/>
-      <c r="W53" s="69"/>
-      <c r="X53" s="69"/>
-      <c r="Y53" s="69"/>
-      <c r="Z53" s="69"/>
+      <c r="B53" s="61"/>
+      <c r="C53" s="60"/>
+      <c r="D53" s="60"/>
+      <c r="E53" s="60"/>
+      <c r="F53" s="60"/>
+      <c r="G53" s="60"/>
+      <c r="H53" s="60"/>
+      <c r="I53" s="60"/>
+      <c r="J53" s="60"/>
+      <c r="K53" s="60"/>
+      <c r="L53" s="60"/>
+      <c r="M53" s="60"/>
+      <c r="N53" s="60"/>
+      <c r="O53" s="60"/>
+      <c r="P53" s="60"/>
+      <c r="Q53" s="60"/>
+      <c r="R53" s="60"/>
+      <c r="S53" s="60"/>
+      <c r="T53" s="60"/>
+      <c r="U53" s="60"/>
+      <c r="V53" s="60"/>
+      <c r="W53" s="60"/>
+      <c r="X53" s="60"/>
+      <c r="Y53" s="60"/>
+      <c r="Z53" s="60"/>
     </row>
     <row r="54" ht="22.5" customHeight="1">
-      <c r="A54" s="68"/>
-      <c r="B54" s="69"/>
-      <c r="C54" s="72" t="s">
+      <c r="A54" s="59"/>
+      <c r="B54" s="60"/>
+      <c r="C54" s="63" t="s">
         <v>132</v>
       </c>
       <c r="G54" s="3"/>
-      <c r="H54" s="69">
+      <c r="H54" s="60">
         <f>COUNTIF($K$14:$K$50,"Xuất sắc")</f>
         <v>1</v>
       </c>
-      <c r="I54" s="69" t="s">
+      <c r="I54" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="J54" s="73">
+      <c r="J54" s="64">
         <f t="shared" ref="J54:J59" si="3">H54/$C$52%</f>
         <v>2.702702703</v>
       </c>
-      <c r="K54" s="69" t="s">
+      <c r="K54" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="L54" s="69"/>
-      <c r="M54" s="69"/>
-      <c r="N54" s="69"/>
-      <c r="O54" s="69"/>
-      <c r="P54" s="69"/>
-      <c r="Q54" s="69"/>
-      <c r="R54" s="69"/>
-      <c r="S54" s="69"/>
-      <c r="T54" s="69"/>
-      <c r="U54" s="69"/>
-      <c r="V54" s="69"/>
-      <c r="W54" s="69"/>
-      <c r="X54" s="69"/>
-      <c r="Y54" s="69"/>
-      <c r="Z54" s="69"/>
+      <c r="L54" s="60"/>
+      <c r="M54" s="60"/>
+      <c r="N54" s="60"/>
+      <c r="O54" s="60"/>
+      <c r="P54" s="60"/>
+      <c r="Q54" s="60"/>
+      <c r="R54" s="60"/>
+      <c r="S54" s="60"/>
+      <c r="T54" s="60"/>
+      <c r="U54" s="60"/>
+      <c r="V54" s="60"/>
+      <c r="W54" s="60"/>
+      <c r="X54" s="60"/>
+      <c r="Y54" s="60"/>
+      <c r="Z54" s="60"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="68"/>
-      <c r="B55" s="69"/>
-      <c r="C55" s="72" t="s">
+      <c r="A55" s="59"/>
+      <c r="B55" s="60"/>
+      <c r="C55" s="63" t="s">
         <v>135</v>
       </c>
       <c r="G55" s="3"/>
-      <c r="H55" s="69">
+      <c r="H55" s="60">
         <f>COUNTIF($K$14:$K$50,"Tốt")</f>
         <v>12</v>
       </c>
-      <c r="I55" s="69" t="s">
+      <c r="I55" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="J55" s="73">
+      <c r="J55" s="64">
         <f t="shared" si="3"/>
         <v>32.43243243</v>
       </c>
-      <c r="K55" s="69" t="s">
+      <c r="K55" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="L55" s="69"/>
-      <c r="M55" s="69"/>
-      <c r="N55" s="69"/>
-      <c r="O55" s="69"/>
-      <c r="P55" s="69"/>
-      <c r="Q55" s="69"/>
-      <c r="R55" s="69"/>
-      <c r="S55" s="69"/>
-      <c r="T55" s="69"/>
-      <c r="U55" s="69"/>
-      <c r="V55" s="69"/>
-      <c r="W55" s="69"/>
-      <c r="X55" s="69"/>
-      <c r="Y55" s="69"/>
-      <c r="Z55" s="69"/>
+      <c r="L55" s="60"/>
+      <c r="M55" s="60"/>
+      <c r="N55" s="60"/>
+      <c r="O55" s="60"/>
+      <c r="P55" s="60"/>
+      <c r="Q55" s="60"/>
+      <c r="R55" s="60"/>
+      <c r="S55" s="60"/>
+      <c r="T55" s="60"/>
+      <c r="U55" s="60"/>
+      <c r="V55" s="60"/>
+      <c r="W55" s="60"/>
+      <c r="X55" s="60"/>
+      <c r="Y55" s="60"/>
+      <c r="Z55" s="60"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="68"/>
-      <c r="B56" s="69"/>
-      <c r="C56" s="72" t="s">
+      <c r="A56" s="59"/>
+      <c r="B56" s="60"/>
+      <c r="C56" s="63" t="s">
         <v>136</v>
       </c>
       <c r="G56" s="3"/>
-      <c r="H56" s="69">
+      <c r="H56" s="60">
         <f>COUNTIF($K$14:$K$50,"Khá")</f>
-        <v>15</v>
-      </c>
-      <c r="I56" s="69" t="s">
+        <v>24</v>
+      </c>
+      <c r="I56" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="J56" s="73">
+      <c r="J56" s="64">
         <f t="shared" si="3"/>
-        <v>40.54054054</v>
-      </c>
-      <c r="K56" s="69" t="s">
+        <v>64.86486486</v>
+      </c>
+      <c r="K56" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="L56" s="69"/>
-      <c r="M56" s="69"/>
-      <c r="N56" s="69"/>
-      <c r="O56" s="69"/>
-      <c r="P56" s="69"/>
-      <c r="Q56" s="69"/>
-      <c r="R56" s="69"/>
-      <c r="S56" s="69"/>
-      <c r="T56" s="69"/>
-      <c r="U56" s="69"/>
-      <c r="V56" s="69"/>
-      <c r="W56" s="69"/>
-      <c r="X56" s="69"/>
-      <c r="Y56" s="69"/>
-      <c r="Z56" s="69"/>
+      <c r="L56" s="60"/>
+      <c r="M56" s="60"/>
+      <c r="N56" s="60"/>
+      <c r="O56" s="60"/>
+      <c r="P56" s="60"/>
+      <c r="Q56" s="60"/>
+      <c r="R56" s="60"/>
+      <c r="S56" s="60"/>
+      <c r="T56" s="60"/>
+      <c r="U56" s="60"/>
+      <c r="V56" s="60"/>
+      <c r="W56" s="60"/>
+      <c r="X56" s="60"/>
+      <c r="Y56" s="60"/>
+      <c r="Z56" s="60"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="68"/>
-      <c r="B57" s="69"/>
-      <c r="C57" s="72" t="s">
+      <c r="A57" s="59"/>
+      <c r="B57" s="60"/>
+      <c r="C57" s="63" t="s">
         <v>137</v>
       </c>
-      <c r="H57" s="69">
+      <c r="H57" s="60">
         <f>COUNTIF($K$14:$K$50,"Trung bình")</f>
-        <v>7</v>
-      </c>
-      <c r="I57" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="I57" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="J57" s="73">
+      <c r="J57" s="64">
         <f t="shared" si="3"/>
-        <v>18.91891892</v>
-      </c>
-      <c r="K57" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="K57" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="L57" s="69"/>
-      <c r="M57" s="69"/>
-      <c r="N57" s="69"/>
-      <c r="O57" s="69"/>
-      <c r="P57" s="69"/>
-      <c r="Q57" s="69"/>
-      <c r="R57" s="69"/>
-      <c r="S57" s="69"/>
-      <c r="T57" s="69"/>
-      <c r="U57" s="69"/>
-      <c r="V57" s="69"/>
-      <c r="W57" s="69"/>
-      <c r="X57" s="69"/>
-      <c r="Y57" s="69"/>
-      <c r="Z57" s="69"/>
+      <c r="L57" s="60"/>
+      <c r="M57" s="60"/>
+      <c r="N57" s="60"/>
+      <c r="O57" s="60"/>
+      <c r="P57" s="60"/>
+      <c r="Q57" s="60"/>
+      <c r="R57" s="60"/>
+      <c r="S57" s="60"/>
+      <c r="T57" s="60"/>
+      <c r="U57" s="60"/>
+      <c r="V57" s="60"/>
+      <c r="W57" s="60"/>
+      <c r="X57" s="60"/>
+      <c r="Y57" s="60"/>
+      <c r="Z57" s="60"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="68"/>
-      <c r="B58" s="69"/>
-      <c r="C58" s="72" t="s">
+      <c r="A58" s="59"/>
+      <c r="B58" s="60"/>
+      <c r="C58" s="63" t="s">
         <v>138</v>
       </c>
-      <c r="D58" s="72"/>
-      <c r="E58" s="72"/>
-      <c r="F58" s="72"/>
+      <c r="D58" s="63"/>
+      <c r="E58" s="63"/>
+      <c r="F58" s="63"/>
       <c r="G58" s="3"/>
-      <c r="H58" s="69">
+      <c r="H58" s="60">
         <f>COUNTIF($K$14:$K$50,"Yếu")</f>
         <v>0</v>
       </c>
-      <c r="I58" s="69" t="s">
+      <c r="I58" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="J58" s="73">
+      <c r="J58" s="64">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K58" s="69" t="s">
+      <c r="K58" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="L58" s="69"/>
-      <c r="M58" s="69"/>
-      <c r="N58" s="69"/>
-      <c r="O58" s="69"/>
-      <c r="P58" s="69"/>
-      <c r="Q58" s="69"/>
-      <c r="R58" s="69"/>
-      <c r="S58" s="69"/>
-      <c r="T58" s="69"/>
-      <c r="U58" s="69"/>
-      <c r="V58" s="69"/>
-      <c r="W58" s="69"/>
-      <c r="X58" s="69"/>
-      <c r="Y58" s="69"/>
-      <c r="Z58" s="69"/>
+      <c r="L58" s="60"/>
+      <c r="M58" s="60"/>
+      <c r="N58" s="60"/>
+      <c r="O58" s="60"/>
+      <c r="P58" s="60"/>
+      <c r="Q58" s="60"/>
+      <c r="R58" s="60"/>
+      <c r="S58" s="60"/>
+      <c r="T58" s="60"/>
+      <c r="U58" s="60"/>
+      <c r="V58" s="60"/>
+      <c r="W58" s="60"/>
+      <c r="X58" s="60"/>
+      <c r="Y58" s="60"/>
+      <c r="Z58" s="60"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="68"/>
-      <c r="B59" s="69"/>
-      <c r="C59" s="72" t="s">
+      <c r="A59" s="59"/>
+      <c r="B59" s="60"/>
+      <c r="C59" s="63" t="s">
         <v>139</v>
       </c>
-      <c r="D59" s="72"/>
-      <c r="E59" s="72"/>
-      <c r="F59" s="72"/>
+      <c r="D59" s="63"/>
+      <c r="E59" s="63"/>
+      <c r="F59" s="63"/>
       <c r="G59" s="3"/>
-      <c r="H59" s="69">
+      <c r="H59" s="60">
         <f>COUNTIF($K$14:$K$50,"Kém")</f>
-        <v>2</v>
-      </c>
-      <c r="I59" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="I59" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="J59" s="73">
+      <c r="J59" s="64">
         <f t="shared" si="3"/>
-        <v>5.405405405</v>
-      </c>
-      <c r="K59" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="K59" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="L59" s="69"/>
-      <c r="M59" s="69"/>
-      <c r="N59" s="69"/>
-      <c r="O59" s="69"/>
-      <c r="P59" s="69"/>
-      <c r="Q59" s="69"/>
-      <c r="R59" s="69"/>
-      <c r="S59" s="69"/>
-      <c r="T59" s="69"/>
-      <c r="U59" s="69"/>
-      <c r="V59" s="69"/>
-      <c r="W59" s="69"/>
-      <c r="X59" s="69"/>
-      <c r="Y59" s="69"/>
-      <c r="Z59" s="69"/>
+      <c r="L59" s="60"/>
+      <c r="M59" s="60"/>
+      <c r="N59" s="60"/>
+      <c r="O59" s="60"/>
+      <c r="P59" s="60"/>
+      <c r="Q59" s="60"/>
+      <c r="R59" s="60"/>
+      <c r="S59" s="60"/>
+      <c r="T59" s="60"/>
+      <c r="U59" s="60"/>
+      <c r="V59" s="60"/>
+      <c r="W59" s="60"/>
+      <c r="X59" s="60"/>
+      <c r="Y59" s="60"/>
+      <c r="Z59" s="60"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="68"/>
+      <c r="A60" s="59"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
@@ -4016,13 +4003,13 @@
     </row>
     <row r="62" ht="21.75" customHeight="1">
       <c r="A62" s="3"/>
-      <c r="B62" s="74"/>
-      <c r="C62" s="74"/>
+      <c r="B62" s="65"/>
+      <c r="C62" s="65"/>
       <c r="D62" s="3"/>
-      <c r="E62" s="75" t="s">
+      <c r="E62" s="66" t="s">
         <v>143</v>
       </c>
-      <c r="I62" s="75" t="s">
+      <c r="I62" s="66" t="s">
         <v>143</v>
       </c>
       <c r="M62" s="3"/>
@@ -4153,14 +4140,14 @@
       <c r="Z66" s="3"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="76" t="s">
+      <c r="A67" s="67" t="s">
         <v>144</v>
       </c>
       <c r="D67" s="3"/>
-      <c r="E67" s="76" t="s">
+      <c r="E67" s="67" t="s">
         <v>145</v>
       </c>
-      <c r="I67" s="76" t="s">
+      <c r="I67" s="67" t="s">
         <v>146</v>
       </c>
       <c r="M67" s="3"/>

</xml_diff>